<commit_message>
Update analysis notebooks and supplementary tables for J Hep submission
- Renumber supplementary tables to the current scheme: S13->S12 (CAGE TSS
  clusters), S14->S13 (per-variant LD + cCRE evidence), S15->S14 (per-dataset
  chromatin evidence), S16->S15 (TF motif disruption).
- Add SpliceAI/Pangolin splice-effect predictions for the 48 LD-expanded
  variants, and the motifbreakR PWM table and motif logos for rs4994910.
- Refresh Fig. 1, 2C, 3, 4, 5B and 5 notebooks and their outputs.
- Update Table S1 (datasets) and the README notebook-to-figure mapping.
- Ignore _backups/.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pppd56wiP5H8NAX6wimSeD
</commit_message>
<xml_diff>
--- a/Table_S1_datasets.xlsx
+++ b/Table_S1_datasets.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-440" yWindow="8760" windowWidth="29400" windowHeight="19120" tabRatio="600" firstSheet="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="33200" yWindow="780" windowWidth="29400" windowHeight="17680" tabRatio="600" firstSheet="14" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -42,21 +42,8 @@
     <font>
       <name val="Arial"/>
       <family val="2"/>
-      <i val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -72,42 +59,8 @@
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
       <sz val="8"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -133,8 +86,22 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -149,18 +116,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B4F8C"/>
-        <bgColor rgb="FF1B4F8C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -168,109 +129,49 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="11" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="35">
     <dxf>
@@ -470,25 +371,25 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <color theme="1"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="general" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <color theme="1"/>
+        <sz val="12"/>
+        <vertAlign val="baseline"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1228,15 +1129,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.95"/>
   <cols>
-    <col width="131.1640625" customWidth="1" style="26" min="1" max="1"/>
-    <col width="42.5" bestFit="1" customWidth="1" style="26" min="2" max="2"/>
-    <col width="49.33203125" bestFit="1" customWidth="1" style="26" min="3" max="3"/>
-    <col width="56.5" bestFit="1" customWidth="1" style="26" min="4" max="4"/>
-    <col width="63.83203125" customWidth="1" style="26" min="5" max="5"/>
-    <col width="55.33203125" bestFit="1" customWidth="1" style="26" min="6" max="6"/>
+    <col width="131.125" customWidth="1" style="18" min="1" max="1"/>
+    <col width="42.5" bestFit="1" customWidth="1" style="18" min="2" max="2"/>
+    <col width="49.375" bestFit="1" customWidth="1" style="18" min="3" max="3"/>
+    <col width="56.5" bestFit="1" customWidth="1" style="18" min="4" max="4"/>
+    <col width="63.875" customWidth="1" style="18" min="5" max="5"/>
+    <col width="55.375" bestFit="1" customWidth="1" style="18" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1246,1293 +1147,1404 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Assay type</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>File identifier</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Figure/panel</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
-        <is>
-          <t>Hannah please insert scRNA-seq here</t>
-        </is>
-      </c>
-      <c r="B4" s="31" t="n"/>
-      <c r="C4" s="31" t="n"/>
-      <c r="D4" s="31" t="n"/>
-      <c r="E4" s="31" t="n"/>
-      <c r="F4" s="31" t="n"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Single-cell + single-nuclei RNA-seq, 19 human liver biopsies (healthy and obese)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>sc/snRNA-seq</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Guilliams et al. 2022 (PMID: 35021063)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>rawData_human.zip; annot_humanAll.csv</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.livercellatlas.org/download.php</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Fig. 2B, Fig. S4A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Hannah please insert scRNA-seq here</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="31" t="n"/>
-      <c r="E5" s="31" t="n"/>
-      <c r="F5" s="31" t="n"/>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Single-nuclei RNA-seq, 47 human liver biopsies from (patients with different stages of metabolic dysfunction-associated steatotic liver disease)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>snRNA-seq</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Gribben et al. 2024 (PMID: 38778114)</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>GSE202379_SeuratObject_AllCells.rds.gz</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE202379</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Fig. S2B, Fig. S4B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM gene/isoform quantification), Huh7.5 cells, SLC38A4 knockout clone KO1 (internal clone ID C12), 6 replicates</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM quantification)</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>This study</t>
         </is>
       </c>
-      <c r="D6" s="36" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>C12_1, C12_2, C12_3, C12_4, C12_5, C12_6</t>
         </is>
       </c>
-      <c r="E6" s="36" t="inlineStr">
-        <is>
-          <t>To be deposited in GEO — accession pending (see note below)</t>
-        </is>
-      </c>
-      <c r="F6" s="36" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE349363</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Fig. 3B–E, Fig. 3H (KO vs WT bars only), Fig. 4B–E</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM gene/isoform quantification), Huh7.5 cells, SLC38A4 knockout clone KO2 (internal clone ID P1.7), 6 replicates</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM quantification)</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>This study</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>P1_7_1, P1_7_2, P1_7_3, P1_7_4, P1_7_5, P1_7_6</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
-        <is>
-          <t>To be deposited in GEO — accession pending (see note below)</t>
-        </is>
-      </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE349363</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Fig. 3B–E, Fig. 3H (KO vs WT bars only), Fig. 4B–E</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM gene/isoform quantification), Huh7.5 cells transfected with a scrambled non-targeting guide RNA (WT control), 6 replicates</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Bulk RNA-seq (RSEM quantification)</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>This study</t>
         </is>
       </c>
-      <c r="D8" s="36" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>SCWT_1, SCWT_2, SCWT_3, SCWT_4, SCWT_5, SCWT_6</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>To be deposited in GEO — accession pending (see note below)</t>
-        </is>
-      </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE349363</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Fig. 3B–E, Fig. 3H (KO vs WT bars only), Fig. 4B–E</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 1</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 1, Male, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>PHH4190-In</t>
-        </is>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>PHH4190</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 2</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 2, Female, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D10" s="36" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>PHH191381</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 3</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 3, Male, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>PHH182851</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 4</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 4, Female, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>PHH183231</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 5</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 5, Male, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D13" s="36" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>PHH180051</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 6</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Bulk ATAC-seq signal, primary human hepatocytes, donor/replicate 6, Female, non-diabetic</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Cebola lab, previously published (PMID: 40452229)</t>
         </is>
       </c>
-      <c r="D14" s="36" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>PHH183001</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>https://ega-archive.org/datasets/EGAD50000001751 (raw data, EGA); https://pubmed.ncbi.nlm.nih.gov/40452229/ (publication)</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
         </is>
       </c>
-      <c r="B15" s="36" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>ENCSR516CPW/ENCFF831BRS</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR516CPW/</t>
         </is>
       </c>
-      <c r="F15" s="36" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (right lobe of liver tissue, male, 45 years)</t>
         </is>
       </c>
-      <c r="B16" s="36" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>ENCSR607BTF/ENCFF646EEM</t>
         </is>
       </c>
-      <c r="E16" s="36" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR607BTF/</t>
         </is>
       </c>
-      <c r="F16" s="36" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (left lobe of liver tissue, female, 61 years)</t>
         </is>
       </c>
-      <c r="B17" s="36" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C17" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>ENCSR624ODL/ENCFF556YQA</t>
         </is>
       </c>
-      <c r="E17" s="36" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR624ODL/</t>
         </is>
       </c>
-      <c r="F17" s="36" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="36" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
         </is>
       </c>
-      <c r="B18" s="36" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C18" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D18" s="36" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>ENCSR685ZMP/ENCFF232QBB</t>
         </is>
       </c>
-      <c r="E18" s="36" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR685ZMP/</t>
         </is>
       </c>
-      <c r="F18" s="36" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (right lobe of liver tissue, male, 40 years)</t>
         </is>
       </c>
-      <c r="B19" s="36" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C19" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>ENCSR836FIL/ENCFF241ZLC</t>
         </is>
       </c>
-      <c r="E19" s="36" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR836FIL/</t>
         </is>
       </c>
-      <c r="F19" s="36" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq signal, adult liver tissue (right lobe of liver tissue female child, 16 years)</t>
         </is>
       </c>
-      <c r="B20" s="36" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Bulk ATAC-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C20" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>ENCSR952SPO/ENCFF469MOB</t>
         </is>
       </c>
-      <c r="E20" s="36" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR952SPO/</t>
         </is>
       </c>
-      <c r="F20" s="36" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A (used to generated pooled track only)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="36" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K4me3, adult liver tissue (right lobe of liver tissue, female, 53 years)</t>
         </is>
       </c>
-      <c r="B21" s="36" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K4me3)</t>
         </is>
       </c>
-      <c r="C21" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>ENCSR344TLI/ENCFF917LFF</t>
         </is>
       </c>
-      <c r="E21" s="36" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR344TLI/</t>
         </is>
       </c>
-      <c r="F21" s="36" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="36" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K4me3, adult liver tissue (liver tissue, male, 31 years)</t>
         </is>
       </c>
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K4me3)</t>
         </is>
       </c>
-      <c r="C22" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D22" s="36" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>ENCSR458WIH/ENCFF053IVC</t>
         </is>
       </c>
-      <c r="E22" s="36" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR458WIH/</t>
         </is>
       </c>
-      <c r="F22" s="36" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="36" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K4me3, adult liver tissue (liver tissue, male, 78 years)</t>
         </is>
       </c>
-      <c r="B23" s="36" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K4me3)</t>
         </is>
       </c>
-      <c r="C23" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D23" s="36" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>ENCSR520BUX/ENCFF962JEC</t>
         </is>
       </c>
-      <c r="E23" s="36" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR520BUX/</t>
         </is>
       </c>
-      <c r="F23" s="36" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="36" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K4me3, adult liver tissue (liver tissue, female, 25 years)</t>
         </is>
       </c>
-      <c r="B24" s="36" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K4me3)</t>
         </is>
       </c>
-      <c r="C24" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D24" s="36" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>ENCSR803JYI/ENCFF280QYJ</t>
         </is>
       </c>
-      <c r="E24" s="36" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR803JYI/</t>
         </is>
       </c>
-      <c r="F24" s="36" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="36" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K27ac, adult liver tissue (liver tissue, male, 31 years)</t>
         </is>
       </c>
-      <c r="B25" s="36" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K27ac)</t>
         </is>
       </c>
-      <c r="C25" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D25" s="36" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>ENCSR230IMS/ENCFF275OLK</t>
         </is>
       </c>
-      <c r="E25" s="36" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR230IMS/</t>
         </is>
       </c>
-      <c r="F25" s="36" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Fig. 5A, Fig. S12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="36" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq of H3K27ac, adult liver tissue (liver tissue with nonobstructive coronary artery disease, male, 32 years)</t>
         </is>
       </c>
-      <c r="B26" s="36" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K27ac)</t>
         </is>
       </c>
-      <c r="C26" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D26" s="36" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>ENCSR458RRZ/ENCFF218ECO</t>
         </is>
       </c>
-      <c r="E26" s="36" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>https://www.encodeproject.org/experiments/ENCSR458RRZ/</t>
         </is>
       </c>
-      <c r="F26" s="36" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Fig. S12; H3K27ac replicated peaks (Methods 5.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq of H3K27ac, adult liver tissue (liver tissue, female, 25 years)</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq (H3K27ac)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR678LND/ENCFF853WPX</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR678LND/</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="36" t="inlineStr">
-        <is>
-          <t>ChIP-seq of H3K27ac, adult liver tissue (liver tissue, female, 25 years)</t>
-        </is>
-      </c>
-      <c r="B27" s="36" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq of H3K27ac, adult liver tissue (right lobe of liver tissue, female, 53 years)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>ChIP-seq (H3K27ac)</t>
         </is>
       </c>
-      <c r="C27" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D27" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR678LND/ENCFF853WPX</t>
-        </is>
-      </c>
-      <c r="E27" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR678LND/</t>
-        </is>
-      </c>
-      <c r="F27" s="36" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR981UJA/ENCFF764VSN</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR981UJA/</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Fig. S12; H3K27ac replicated peaks (Methods 5.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq of H3K27ac, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq (H3K27ac)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR864OOO</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR864OOO/</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>H3K27ac replicated peaks (Methods 5.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq of H3K27ac, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>ChIP-seq (H3K27ac)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR779ISJ</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR779ISJ/</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>H3K27ac replicated peaks (Methods 5.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (left lobe of liver tissue, male, 45 years)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF065AJK</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF065AJK/</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, male, 45 years)</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF152MZM</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF152MZM/</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF253OSP</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF253OSP/</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF321WIO</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF321WIO/</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years) 1</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF481ZPW</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF481ZPW/</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years) 2</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq (signal, minus strand)</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>ENCFF776YAA</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/files/ENCFF776YAA/</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 1</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>CAGE (CTSS, individual donor)</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>CNhs12340</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor1.CNhs12340.11523-119I2.hg38.nobarcode.ctss.bed.gz</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 2</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>CAGE (CTSS, individual donor)</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>CNhs12349</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor2.CNhs12349.11603-120I1.hg38.nobarcode.ctss.bed.gz</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 3</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>CAGE (CTSS, individual donor)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>CNhs12626</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor3.CNhs12626.11684-122I1.hg38.nobarcode.ctss.bed.gz</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5 CAGE (CTSS) data, liver, adult, pooled donor sample (pool1; mixed sex, ages 64/69/70)</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>CAGE (CTSS, pooled tissue)</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>FANTOM5</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>CNhs10624 (FF:10018-101C9)</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.tissue.hCAGE/liver%252c%2520adult%252c%2520pool1.CNhs10624.10018-101C9.hg38.nobarcode.ctss.bed.gz</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Bulk DNase-seq (signal, individual replicate)</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR164TBP/ENCFF634BMR</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR164TBP/</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="36" t="inlineStr">
-        <is>
-          <t>ChIP-seq of H3K27ac, adult liver tissue (right lobe of liver tissue, female, 53 years)</t>
-        </is>
-      </c>
-      <c r="B28" s="36" t="inlineStr">
-        <is>
-          <t>ChIP-seq (H3K27ac)</t>
-        </is>
-      </c>
-      <c r="C28" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D28" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR981UJA/ENCFF764VSN</t>
-        </is>
-      </c>
-      <c r="E28" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR981UJA/</t>
-        </is>
-      </c>
-      <c r="F28" s="36" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, male, 45 years)</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Bulk DNase-seq (signal, individual replicate)</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR628NEA/ENCFF606YDZ</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR628NEA/</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (left lobe of liver tissue, male, 45 years)</t>
-        </is>
-      </c>
-      <c r="B29" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C29" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D29" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF065AJK</t>
-        </is>
-      </c>
-      <c r="E29" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF065AJK/</t>
-        </is>
-      </c>
-      <c r="F29" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, male, 45 years)</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C30" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D30" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF152MZM</t>
-        </is>
-      </c>
-      <c r="E30" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF152MZM/</t>
-        </is>
-      </c>
-      <c r="F30" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
-        </is>
-      </c>
-      <c r="B31" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C31" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D31" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF253OSP</t>
-        </is>
-      </c>
-      <c r="E31" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF253OSP/</t>
-        </is>
-      </c>
-      <c r="F31" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
-        </is>
-      </c>
-      <c r="B32" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C32" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D32" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF321WIO</t>
-        </is>
-      </c>
-      <c r="E32" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF321WIO/</t>
-        </is>
-      </c>
-      <c r="F32" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years) 1</t>
-        </is>
-      </c>
-      <c r="B33" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C33" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D33" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF481ZPW</t>
-        </is>
-      </c>
-      <c r="E33" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF481ZPW/</t>
-        </is>
-      </c>
-      <c r="F33" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years) 2</t>
-        </is>
-      </c>
-      <c r="B34" s="36" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq (signal, minus strand)</t>
-        </is>
-      </c>
-      <c r="C34" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D34" s="36" t="inlineStr">
-        <is>
-          <t>ENCFF776YAA</t>
-        </is>
-      </c>
-      <c r="E34" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/files/ENCFF776YAA/</t>
-        </is>
-      </c>
-      <c r="F34" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 1</t>
-        </is>
-      </c>
-      <c r="B35" s="36" t="inlineStr">
-        <is>
-          <t>CAGE (CTSS, individual donor)</t>
-        </is>
-      </c>
-      <c r="C35" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5</t>
-        </is>
-      </c>
-      <c r="D35" s="36" t="inlineStr">
-        <is>
-          <t>CNhs12340</t>
-        </is>
-      </c>
-      <c r="E35" s="36" t="inlineStr">
-        <is>
-          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor1.CNhs12340.11523-119I2.hg38.nobarcode.ctss.bed.gz</t>
-        </is>
-      </c>
-      <c r="F35" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 2</t>
-        </is>
-      </c>
-      <c r="B36" s="36" t="inlineStr">
-        <is>
-          <t>CAGE (CTSS, individual donor)</t>
-        </is>
-      </c>
-      <c r="C36" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5</t>
-        </is>
-      </c>
-      <c r="D36" s="36" t="inlineStr">
-        <is>
-          <t>CNhs12349</t>
-        </is>
-      </c>
-      <c r="E36" s="36" t="inlineStr">
-        <is>
-          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor2.CNhs12349.11603-120I1.hg38.nobarcode.ctss.bed.gz</t>
-        </is>
-      </c>
-      <c r="F36" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5 CAGE (CTSS) data, primary human hepatocyte, donor 3</t>
-        </is>
-      </c>
-      <c r="B37" s="36" t="inlineStr">
-        <is>
-          <t>CAGE (CTSS, individual donor)</t>
-        </is>
-      </c>
-      <c r="C37" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5</t>
-        </is>
-      </c>
-      <c r="D37" s="36" t="inlineStr">
-        <is>
-          <t>CNhs12626</t>
-        </is>
-      </c>
-      <c r="E37" s="36" t="inlineStr">
-        <is>
-          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.primary_cell.hCAGE/Hepatocyte%252c%2520donor3.CNhs12626.11684-122I1.hg38.nobarcode.ctss.bed.gz</t>
-        </is>
-      </c>
-      <c r="F37" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5 CAGE (CTSS) data, liver, adult, pooled donor sample (pool1; mixed sex, ages 64/69/70)</t>
-        </is>
-      </c>
-      <c r="B38" s="36" t="inlineStr">
-        <is>
-          <t>CAGE (CTSS, pooled tissue)</t>
-        </is>
-      </c>
-      <c r="C38" s="36" t="inlineStr">
-        <is>
-          <t>FANTOM5</t>
-        </is>
-      </c>
-      <c r="D38" s="36" t="inlineStr">
-        <is>
-          <t>CNhs10624 (FF:10018-101C9)</t>
-        </is>
-      </c>
-      <c r="E38" s="36" t="inlineStr">
-        <is>
-          <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_latest/basic/human.tissue.hCAGE/liver%252c%2520adult%252c%2520pool1.CNhs10624.10018-101C9.hg38.nobarcode.ctss.bed.gz</t>
-        </is>
-      </c>
-      <c r="F38" s="36" t="inlineStr">
-        <is>
-          <t>Fig. 5A, Fig. S12 (isoform selection; not shown as a track)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="36" t="inlineStr">
-        <is>
-          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 47 years)</t>
-        </is>
-      </c>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>DNase-seq signal, adult liver tissue (left lobe of liver tissue, male, 45 years)</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>Bulk DNase-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C39" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D39" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR164TBP/ENCFF634BMR</t>
-        </is>
-      </c>
-      <c r="E39" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR164TBP/</t>
-        </is>
-      </c>
-      <c r="F39" s="36" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR802ZYE/ENCFF412PVV</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR802ZYE/</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="36" t="inlineStr">
-        <is>
-          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, male, 45 years)</t>
-        </is>
-      </c>
-      <c r="B40" s="36" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years)</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Bulk DNase-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C40" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D40" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR628NEA/ENCFF606YDZ</t>
-        </is>
-      </c>
-      <c r="E40" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR628NEA/</t>
-        </is>
-      </c>
-      <c r="F40" s="36" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR909HFI/ENCFF020EPF</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR909HFI/</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="36" t="inlineStr">
-        <is>
-          <t>DNase-seq signal, adult liver tissue (left lobe of liver tissue, male, 45 years)</t>
-        </is>
-      </c>
-      <c r="B41" s="36" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>Bulk DNase-seq (signal, individual replicate)</t>
         </is>
       </c>
-      <c r="C41" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D41" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR802ZYE/ENCFF412PVV</t>
-        </is>
-      </c>
-      <c r="E41" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR802ZYE/</t>
-        </is>
-      </c>
-      <c r="F41" s="36" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>ENCODE</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>ENCSR933GMM/ENCFF082KAC</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>https://www.encodeproject.org/experiments/ENCSR933GMM/</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>Fig. S12</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="36" t="inlineStr">
-        <is>
-          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 53 years)</t>
-        </is>
-      </c>
-      <c r="B42" s="36" t="inlineStr">
-        <is>
-          <t>Bulk DNase-seq (signal, individual replicate)</t>
-        </is>
-      </c>
-      <c r="C42" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D42" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR909HFI/ENCFF020EPF</t>
-        </is>
-      </c>
-      <c r="E42" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR909HFI/</t>
-        </is>
-      </c>
-      <c r="F42" s="36" t="inlineStr">
-        <is>
-          <t>Fig. S12</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="36" t="inlineStr">
-        <is>
-          <t>DNase-seq signal, adult liver tissue (right lobe of liver tissue, female, 41 years)</t>
-        </is>
-      </c>
-      <c r="B43" s="36" t="inlineStr">
-        <is>
-          <t>Bulk DNase-seq (signal, individual replicate)</t>
-        </is>
-      </c>
-      <c r="C43" s="36" t="inlineStr">
-        <is>
-          <t>ENCODE</t>
-        </is>
-      </c>
-      <c r="D43" s="36" t="inlineStr">
-        <is>
-          <t>ENCSR933GMM/ENCFF082KAC</t>
-        </is>
-      </c>
-      <c r="E43" s="36" t="inlineStr">
-        <is>
-          <t>https://www.encodeproject.org/experiments/ENCSR933GMM/</t>
-        </is>
-      </c>
-      <c r="F43" s="36" t="inlineStr">
-        <is>
-          <t>Fig. S12</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="36" t="inlineStr">
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>* All datasets in this table are on genome assembly GRCh38/hg38.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="36" t="inlineStr">
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>ENCSR373TDL (ATAC-seq) and ENCSR795VEN (H3K4me3) were excluded for low signal.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>